<commit_message>
chore: record GitHub outreach and community gates
</commit_message>
<xml_diff>
--- a/Table.xlsx
+++ b/Table.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link Submit" sheetId="1" r:id="Ra2525b19ec964dd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OldPhotoLive AI" sheetId="2" r:id="R4295dfd96d5f4e25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RainbowPetAI" sheetId="3" r:id="R19a66602c97e4d12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RspAI" sheetId="4" r:id="R01eedcb7c09d4350"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison Text" sheetId="5" r:id="Re6784c7c048b4e0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graffiti Name AI" sheetId="6" r:id="R14c688d2171f4e29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Log" sheetId="7" r:id="R2f7f5960b4bc4d46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KGR &lt; 0.25长尾词候选表" sheetId="8" r:id="R38b5d9720c5a4912"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link Submit" sheetId="1" r:id="R55adf86a2c7a4c68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OldPhotoLive AI" sheetId="2" r:id="Rb56fef919018474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RainbowPetAI" sheetId="3" r:id="R65e54b1c2ead46d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RspAI" sheetId="4" r:id="R8b4d85086064476f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison Text" sheetId="5" r:id="Rd6f583975e344ae5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graffiti Name AI" sheetId="6" r:id="R368bb178f67d4729"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Log" sheetId="7" r:id="R3f1c8665a3094761"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KGR &lt; 0.25长尾词候选表" sheetId="8" r:id="R9de92f2bd7d04b2b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1198,7 +1198,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="42">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -1331,6 +1331,37 @@
     <x:xf numFmtId="200" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1412,7 +1443,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R270f3f35bf5c48a3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rebe7d277c8ba4513"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1444,7 +1475,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3704cc4436924f50"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R60e08f0cf2044b2f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2552,16 +2583,60 @@
       <x:c r="F58" s="23"/>
     </x:row>
     <x:row r="59" ht="18" customHeight="1">
-      <x:c r="A59" s="30"/>
-      <x:c r="B59" s="37"/>
+      <x:c r="A59" s="44" t="str">
+        <x:v>https://github.com/Syndred/pet-memorial-resources</x:v>
+      </x:c>
+      <x:c r="B59" s="45" t="str">
+        <x:v>RainbowPetAI</x:v>
+      </x:c>
+      <x:c r="C59" s="46" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D59" s="47" t="n">
+        <x:v>46240</x:v>
+      </x:c>
+      <x:c r="E59" s="48" t="str">
+        <x:v>公开资源仓库已创建；README 含真实宠物离世支持资源、纪念清单、隐私建议、RainbowPetAI 链接和展示图；公开页面与链接已验收。</x:v>
+      </x:c>
+      <x:c r="F59" s="48" t="str">
+        <x:v>https://github.com/Syndred/pet-memorial-resources</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="18" customHeight="1">
-      <x:c r="A60" s="30"/>
-      <x:c r="B60" s="37"/>
+      <x:c r="A60" s="44" t="str">
+        <x:v>https://www.indiehackers.com/new-post</x:v>
+      </x:c>
+      <x:c r="B60" s="45" t="str">
+        <x:v>RainbowPetAI</x:v>
+      </x:c>
+      <x:c r="C60" s="46" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D60" s="47" t="n">
+        <x:v>46240</x:v>
+      </x:c>
+      <x:c r="E60" s="48" t="str">
+        <x:v>@Syndred 已登录，但平台显示 You can't create posts yet；需真实社区互动并获管理员解锁，或付费 IH Plus。本轮不付费、不制造互动。</x:v>
+      </x:c>
+      <x:c r="F60" s="48" t="str"/>
     </x:row>
     <x:row r="61" ht="18" customHeight="1">
-      <x:c r="A61" s="30"/>
-      <x:c r="B61" s="37"/>
+      <x:c r="A61" s="44" t="str">
+        <x:v>https://news.ycombinator.com/</x:v>
+      </x:c>
+      <x:c r="B61" s="45" t="str">
+        <x:v>RainbowPetAI</x:v>
+      </x:c>
+      <x:c r="C61" s="46" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D61" s="47" t="n">
+        <x:v>46240</x:v>
+      </x:c>
+      <x:c r="E61" s="48" t="str">
+        <x:v>用户于 2026-08-06 取消 Hacker News 提交：没有账号，不再处理。</x:v>
+      </x:c>
+      <x:c r="F61" s="48" t="str"/>
     </x:row>
     <x:row r="62" ht="18" customHeight="1">
       <x:c r="A62" s="30"/>
@@ -6357,18 +6432,18 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="Rb18ecfd43d9a4b42"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="R82c0116299054be0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="Red298e4f20fa416e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="R42a8230a0ed74ba8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="R732ad9ad67f343d5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="Rcce07a585ff34cf2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="R33993842fb1645ec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="Re4594f0a15bd4845"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="R254b40a1f39a4748"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="R7892850d3f00493f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="Rc86c4fe2ceee4d6c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="Rd215e10ee6e04a70"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="R17d9ffd82e9d434f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="Rdf46d60dd1ea4610"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="R5ac2e38e86454d35"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="Rf8f2ef70b0f94a63"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0da738b31dd64eee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61a856b478c54d93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9689,12 +9764,12 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="R831124cd34644ae5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="Re387f1edce084c2b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="R066844ace5fd4426"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="R90cd20c24f28411b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="R60e94a8e3a9240d9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="Rd4e5900384a04544"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="R0a4b9bc74993426e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="R515e735bc8b544ff"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="R2e67d3847a03409b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="R81c45f8ee2e74cfc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="Ra969f2e654934d50"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="R1ec36f98c74046c2"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -13010,13 +13085,13 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="Re47b4a9f53704664"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="R84c3eb3fab5541dd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="Rffba2d8f273a445e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="R8611042aeed94fa5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="R86b373ef37634777"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="R9a80854b315945d8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="R0d6d701ccbd54fc8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="R67c60d086a304fb7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="Reef2abeda311408b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="R00f428367ac344ce"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="Rbd9db1171d36477e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="Rb6980a7890a24d44"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="R1006a57f99364596"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="R3b909c09702a49be"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -16330,13 +16405,13 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="Rfdccfbd7b25e45b7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="R24f071a4325444bc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="R9e057f384bba44a5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="R859ac806e9f34dce"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="R99c0eb13d5b84988"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="R6f84dceba1da406b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="R2cff37e548474fb6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="R338a140e4b464986"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="Rea6d0d87de6941bd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="R67431caf0ff7416f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="R8d324a8a74a24de4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="R529c3fc8334d4d80"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="R0886b29a5f0d4794"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="Rcc5886cf202c4619"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -19654,7 +19729,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8279e68be7be4f2f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40e81d39e8834eb0"/>
 </x:worksheet>
 </file>
 
@@ -21046,7 +21121,7 @@
     <x:row r="1000" ht="18" customHeight="1"/>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc242372b4ff34e74"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ff3521535a5425d"/>
 </x:worksheet>
 </file>
 
@@ -21180,7 +21255,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0267c1fb90e44369"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1aa90d3263304bbc"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>